<commit_message>
Auto Candidate IDs; simpler interview form
- New candidates get the next ID after the most recently added one
  (C030 -> C031, same prefix and padding); Excel rows without an ID
  are numbered in row order, and the preview shows the range. The
  template's Candidate ID column is now optional.
- Interview form: ชื่อโครงการ / หมายเหตุ removed (existing values kept);
  the location field now really hides for online interviews (.field's
  display:flex was overriding [hidden]) and online/onsite each send
  only their own place or link.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/candidate-import-template.xlsx
+++ b/templates/candidate-import-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\101840\AppData\Local\Claude-Data\claude_pzs8sxrjxfjjc\scratch-workspaces\935a3153-45e9-4dc8-86a4-cc9d0bd8a24e\944adfba-1422-4e02-bf6e-de6f8e99ffd7\scratch-2026-10-26-3f28e8\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D815ECEC-81BE-4525-B40B-3D0AD864A1DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2EE9DA8B-9F0F-47FD-8AD8-448014D0EA7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3588" yWindow="2412" windowWidth="17280" windowHeight="9828" xr2:uid="{E9CDE7A6-FC68-4347-B3A2-1240FD20A2F5}"/>
+    <workbookView xWindow="3588" yWindow="2412" windowWidth="17280" windowHeight="9828" xr2:uid="{D183583B-7B45-4918-AE9E-C4E846BD9B2F}"/>
   </bookViews>
   <sheets>
     <sheet name="Candidate Database" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="142">
   <si>
     <t>Template นำเข้าผู้สมัคร · Candidate Pool</t>
   </si>
@@ -55,21 +55,12 @@
     <t>สถานะและนัดสัมภาษณ์ (ไม่บังคับ)</t>
   </si>
   <si>
-    <t>★ ต้องกรอก · รหัสผู้สมัคร ห้ามซ้ำกันในไฟล์ ถ้าตรงกับรหัสที่มีในระบบแล้ว ข้อมูลในไฟล์จะแทนที่ข้อมูลเดิมของคนนั้น</t>
+    <t>เว้นว่าง = ระบบรันรหัสให้อัตโนมัติต่อจากผู้สมัครคนล่าสุด ตามลำดับแถว · ใส่รหัสที่มีในระบบแล้ว = อัปเดตข้อมูลของคนนั้นแทนที่ของเดิม</t>
   </si>
   <si>
     <t>Candidate ID</t>
   </si>
   <si>
-    <t>EX-001</t>
-  </si>
-  <si>
-    <t>EX-002</t>
-  </si>
-  <si>
-    <t>EX-003</t>
-  </si>
-  <si>
     <t>★ ต้องกรอก · ชื่อและนามสกุลเต็มของผู้สมัคร</t>
   </si>
   <si>
@@ -325,7 +316,7 @@
     <t>ก่อนนำเข้า</t>
   </si>
   <si>
-    <t>ลบ 3 แถวตัวอย่างสีเขียว (EX-001 ถึง EX-003) ออก แล้วบันทึกเป็น .xlsx</t>
+    <t>ลบ 3 แถวตัวอย่างสีเขียวออก แล้วบันทึกเป็น .xlsx (ถ้าลืม ระบบจะเพิ่มผู้สมัครตัวอย่าง 3 คนเข้าไปจริง)</t>
   </si>
   <si>
     <t>นำเข้าอย่างไร</t>
@@ -343,19 +334,19 @@
     <t>ต้องกรอก</t>
   </si>
   <si>
-    <t>Candidate ID และ ชื่อ-นามสกุล แถวที่ขาดอย่างใดอย่างหนึ่งจะถูกข้าม</t>
+    <t>ชื่อ-นามสกุล แถวที่ไม่มีชื่อจะถูกข้าม · Candidate ID เว้นว่างได้ ระบบรันให้ (เช่น คนล่าสุด C030 แถวแรกจะได้ C031 แถวถัดไป C032)</t>
   </si>
   <si>
     <t>รหัสซ้ำ</t>
   </si>
   <si>
-    <t>ถ้า Candidate ID ซ้ำกันในไฟล์ ระบบจะแจ้งเตือนและข้ามแถวที่ซ้ำ · ถ้าตรงกับผู้สมัครที่มีในระบบแล้ว ข้อมูลในไฟล์จะแทนที่ของเดิมทั้งแถว รวมถึงคะแนนรายมิติ (ช่องคะแนนที่เว้นว่างจะกลายเป็นยังไม่ให้คะแนน)</t>
+    <t>ถ้าใส่ Candidate ID ซ้ำกันในไฟล์ ระบบจะแจ้งเตือนและข้ามแถวที่ซ้ำ · ถ้าตรงกับผู้สมัครที่มีในระบบแล้ว ข้อมูลในไฟล์จะแทนที่ของเดิมทั้งแถว รวมถึงคะแนนรายมิติ (ช่องคะแนนที่เว้นว่างจะกลายเป็นยังไม่ให้คะแนน)</t>
   </si>
   <si>
     <t>Candidate Score</t>
   </si>
   <si>
-    <t>ไม่ต้องกรอก ระบบคำนวณจากคะแนน 7 มิติ = ผลรวมคะแนน ÷ (5 × จำนวนมิติที่ให้คะแนน) × 100 · ตัวอย่าง EX-001 = 31 ÷ 35 = 89%</t>
+    <t>ไม่ต้องกรอก ระบบคำนวณจากคะแนน 7 มิติ = ผลรวมคะแนน ÷ (5 × จำนวนมิติที่ให้คะแนน) × 100 · ตัวอย่างแถวแรก (สมชาย) = 31 ÷ 35 = 89%</t>
   </si>
   <si>
     <t>คะแนนรายมิติ</t>
@@ -391,13 +382,13 @@
     <t>คำอธิบาย</t>
   </si>
   <si>
-    <t>ตัวอย่าง (EX-001)</t>
+    <t>ตัวอย่าง (แถวแรก)</t>
   </si>
   <si>
     <t>ข้อความ</t>
   </si>
   <si>
-    <t>รหัสผู้สมัคร ห้ามซ้ำกันในไฟล์ ถ้าตรงกับรหัสที่มีในระบบแล้ว ข้อมูลในไฟล์จะแทนที่ข้อมูลเดิมของคนนั้น</t>
+    <t/>
   </si>
   <si>
     <t>ชื่อและนามสกุลเต็มของผู้สมัคร</t>
@@ -461,9 +452,6 @@
   </si>
   <si>
     <t>วันที่และเวลา</t>
-  </si>
-  <si>
-    <t/>
   </si>
 </sst>
 </file>
@@ -688,10 +676,10 @@
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -727,10 +715,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1046,7 +1034,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96B4AEF7-4026-45B7-A134-2B8CF5B0258E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EA8370A-34DA-4835-BCDA-B0F08EDC4176}">
   <dimension ref="A1:AB500"/>
   <sheetFormatPr defaultRowHeight="16.8"/>
   <cols>
@@ -1157,188 +1145,186 @@
         <v>9</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="M5" s="15" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="N5" s="15" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="O5" s="15" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="P5" s="15" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="Q5" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="R5" s="15" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="S5" s="15" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="T5" s="15" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="U5" s="15" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="V5" s="15" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="W5" s="15" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="X5" s="15" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="Y5" s="15" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="Z5" s="15" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AA5" s="15" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="AB5" s="15" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:28" ht="49.95" customHeight="1">
       <c r="A6" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="G6" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="H6" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="I6" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="J6" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="K6" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="L6" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="M6" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="N6" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="O6" s="17" t="s">
-        <v>64</v>
-      </c>
-      <c r="P6" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q6" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="R6" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="S6" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="T6" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="U6" s="17" t="s">
-        <v>79</v>
-      </c>
-      <c r="V6" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="W6" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="X6" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="Y6" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="Z6" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="AA6" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="AB6" s="17" t="s">
-        <v>95</v>
+      <c r="B6" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="J6" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="K6" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="L6" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="M6" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N6" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="O6" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="P6" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q6" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="R6" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="S6" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="T6" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="U6" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="V6" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="W6" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="X6" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y6" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="Z6" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="AA6" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="AB6" s="16" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:28" ht="48" customHeight="1">
-      <c r="A7" s="18" t="s">
-        <v>11</v>
-      </c>
+      <c r="A7" s="18"/>
       <c r="B7" s="18" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F7" s="19">
         <v>32</v>
@@ -1347,13 +1333,13 @@
         <v>8</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="I7" s="18" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K7" s="20">
         <v>45000</v>
@@ -1365,10 +1351,10 @@
         <v>46315</v>
       </c>
       <c r="N7" s="19" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="O7" s="18" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="P7" s="19">
         <v>5</v>
@@ -1392,7 +1378,7 @@
         <v>5</v>
       </c>
       <c r="W7" s="19" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="X7" s="22"/>
       <c r="Y7" s="18"/>
@@ -1401,20 +1387,18 @@
       <c r="AB7" s="18"/>
     </row>
     <row r="8" spans="1:28" ht="48" customHeight="1">
-      <c r="A8" s="18" t="s">
-        <v>12</v>
-      </c>
+      <c r="A8" s="18"/>
       <c r="B8" s="18" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F8" s="19">
         <v>28</v>
@@ -1423,13 +1407,13 @@
         <v>5</v>
       </c>
       <c r="H8" s="18" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="I8" s="18" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="J8" s="18" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="K8" s="20">
         <v>32000</v>
@@ -1441,10 +1425,10 @@
         <v>46317</v>
       </c>
       <c r="N8" s="19" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="O8" s="18" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="P8" s="19">
         <v>4</v>
@@ -1468,7 +1452,7 @@
         <v>3</v>
       </c>
       <c r="W8" s="19" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="X8" s="22"/>
       <c r="Y8" s="18"/>
@@ -1477,20 +1461,18 @@
       <c r="AB8" s="18"/>
     </row>
     <row r="9" spans="1:28" ht="48" customHeight="1">
-      <c r="A9" s="18" t="s">
-        <v>13</v>
-      </c>
+      <c r="A9" s="18"/>
       <c r="B9" s="18" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F9" s="19">
         <v>35</v>
@@ -1499,10 +1481,10 @@
         <v>10</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="I9" s="18" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="J9" s="18"/>
       <c r="K9" s="20">
@@ -1515,10 +1497,10 @@
         <v>46318</v>
       </c>
       <c r="N9" s="19" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O9" s="18" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="P9" s="19">
         <v>3</v>
@@ -1542,14 +1524,14 @@
         <v>2</v>
       </c>
       <c r="W9" s="19" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="X9" s="22"/>
       <c r="Y9" s="18"/>
       <c r="Z9" s="18"/>
       <c r="AA9" s="18"/>
       <c r="AB9" s="18" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:28">
@@ -10893,84 +10875,84 @@
     <mergeCell ref="A4:M4"/>
   </mergeCells>
   <dataValidations count="28">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Candidate ID" prompt="★ ต้องกรอก · รหัสผู้สมัคร ห้ามซ้ำกันในไฟล์ ถ้าตรงกับรหัสที่มีในระบบแล้ว ข้อมูลในไฟล์จะแทนที่ข้อมูลเดิมของคนนั้น" sqref="A7:A500" xr:uid="{4ACEA1BF-6F52-4337-B816-6BA43DB51452}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="ชื่อ-นามสกุล" prompt="★ ต้องกรอก · ชื่อและนามสกุลเต็มของผู้สมัคร" sqref="B7:B500" xr:uid="{5A040B30-CBF4-4B2C-BC40-D84BC7718070}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Email" prompt="อีเมลผู้สมัคร · เห็นเฉพาะ HRS แผนกไม่เห็น" sqref="C7:C500" xr:uid="{0C58AF19-FBC1-4A0B-8716-E92FC6943A47}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="เบอร์โทรศัพท์" prompt="เบอร์ติดต่อผู้สมัคร พิมพ์ได้ทั้ง 0812345678 หรือ 081-234-5678 · เห็นเฉพาะ HRS แผนกไม่เห็น" sqref="D7:D500" xr:uid="{C531D425-DDBB-4A4C-85A1-D1D4B1B6735D}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="ตำแหน่ง" prompt="ตำแหน่งที่สมัคร ระบบใช้จัดกลุ่มและกรอง พิมพ์ชื่อตำแหน่งให้เหมือนกันทุกแถว" sqref="E7:E500" xr:uid="{C69C5C22-3E66-408A-8D44-26675A3DA3BB}"/>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่อายุเป็นตัวเลข 15 ถึง 80" promptTitle="อายุ" prompt="ตัวเลขเท่านั้น (ปี)" sqref="F7:F500" xr:uid="{0B5B01B5-5AA8-4C68-8B1D-93473B1600D7}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Candidate ID" prompt="เว้นว่าง = ระบบรันรหัสให้อัตโนมัติต่อจากผู้สมัครคนล่าสุด ตามลำดับแถว · ใส่รหัสที่มีในระบบแล้ว = อัปเดตข้อมูลของคนนั้นแทนที่ของเดิม" sqref="A7:A500" xr:uid="{031AF327-2E18-4488-8199-12B61F871D77}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="ชื่อ-นามสกุล" prompt="★ ต้องกรอก · ชื่อและนามสกุลเต็มของผู้สมัคร" sqref="B7:B500" xr:uid="{3507AE42-B65F-41C9-9737-4BB13D8FDD61}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Email" prompt="อีเมลผู้สมัคร · เห็นเฉพาะ HRS แผนกไม่เห็น" sqref="C7:C500" xr:uid="{B12C2A90-E301-4F36-974D-6C55219A46DC}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="เบอร์โทรศัพท์" prompt="เบอร์ติดต่อผู้สมัคร พิมพ์ได้ทั้ง 0812345678 หรือ 081-234-5678 · เห็นเฉพาะ HRS แผนกไม่เห็น" sqref="D7:D500" xr:uid="{236E182E-16C0-4C8A-9DD5-D6C30C9D6CE0}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="ตำแหน่ง" prompt="ตำแหน่งที่สมัคร ระบบใช้จัดกลุ่มและกรอง พิมพ์ชื่อตำแหน่งให้เหมือนกันทุกแถว" sqref="E7:E500" xr:uid="{574F9FAA-BB86-4023-B31A-4329345127C9}"/>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่อายุเป็นตัวเลข 15 ถึง 80" promptTitle="อายุ" prompt="ตัวเลขเท่านั้น (ปี)" sqref="F7:F500" xr:uid="{49DD95C7-0655-4A31-9660-6076A1EB45EB}">
       <formula1>15</formula1>
       <formula2>80</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลข 0 ถึง 60" promptTitle="ประสบการณ์รวม (ปี)" prompt="ตัวเลขเท่านั้น ใส่ทศนิยมได้ เช่น 5.5" sqref="G7:G500" xr:uid="{8EA140EC-0805-4601-A363-88D704068446}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลข 0 ถึง 60" promptTitle="ประสบการณ์รวม (ปี)" prompt="ตัวเลขเท่านั้น ใส่ทศนิยมได้ เช่น 5.5" sqref="G7:G500" xr:uid="{5EC2C860-8268-404A-BC18-7F3EB3B403E6}">
       <formula1>0</formula1>
       <formula2>60</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="การศึกษา" prompt="วุฒิสูงสุด สาขา และสถาบัน" sqref="H7:H500" xr:uid="{38D7E969-5859-4E48-8B2D-5C046A955727}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="บริษัทล่าสุด" prompt="ชื่อบริษัทที่ทำงานล่าสุด" sqref="I7:I500" xr:uid="{174533A2-D022-4659-AC72-0BEB9CF4817B}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Resume/CV" prompt="ลิงก์ไฟล์ Resume / CV ต้องขึ้นต้นด้วย https:// (เช่น ลิงก์ Google Drive หรือ SharePoint ที่เปิดสิทธิ์ให้แผนกดูได้)" sqref="J7:J500" xr:uid="{05DFDD76-3A8E-4116-8ACB-64D4F6E2EDA5}"/>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขเท่านั้น ไม่ต้องพิมพ์ , หรือ ฿" promptTitle="เงินเดือนปัจจุบัน" prompt="ตัวเลขเท่านั้น (บาท/เดือน) ไม่ต้องพิมพ์ ฿ · แผนกจะยังไม่เห็นเงินเดือนจนกว่า HRS เปิดให้เห็นรายคนในระบบ" sqref="K7:K500" xr:uid="{6E58B46F-CE50-4045-87D3-95324882AAFF}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="การศึกษา" prompt="วุฒิสูงสุด สาขา และสถาบัน" sqref="H7:H500" xr:uid="{1D6CF2A0-FB01-484A-8446-1F36D293F44A}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="บริษัทล่าสุด" prompt="ชื่อบริษัทที่ทำงานล่าสุด" sqref="I7:I500" xr:uid="{1764D736-5D8F-4175-94AE-506A62C21B14}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Resume/CV" prompt="ลิงก์ไฟล์ Resume / CV ต้องขึ้นต้นด้วย https:// (เช่น ลิงก์ Google Drive หรือ SharePoint ที่เปิดสิทธิ์ให้แผนกดูได้)" sqref="J7:J500" xr:uid="{6648D02C-AE3A-49C9-B503-D3E8EAC5F1D3}"/>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขเท่านั้น ไม่ต้องพิมพ์ , หรือ ฿" promptTitle="เงินเดือนปัจจุบัน" prompt="ตัวเลขเท่านั้น (บาท/เดือน) ไม่ต้องพิมพ์ ฿ · แผนกจะยังไม่เห็นเงินเดือนจนกว่า HRS เปิดให้เห็นรายคนในระบบ" sqref="K7:K500" xr:uid="{82B870D8-BCA5-40B5-99F1-6EBE73450677}">
       <formula1>0</formula1>
       <formula2>10000000</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขเท่านั้น ไม่ต้องพิมพ์ , หรือ ฿" promptTitle="เงินเดือนคาดหวัง" prompt="ตัวเลขเท่านั้น (บาท/เดือน) ไม่ต้องพิมพ์ ฿" sqref="L7:L500" xr:uid="{66FCEEB7-12F0-49FD-9F11-A54986818DEB}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขเท่านั้น ไม่ต้องพิมพ์ , หรือ ฿" promptTitle="เงินเดือนคาดหวัง" prompt="ตัวเลขเท่านั้น (บาท/เดือน) ไม่ต้องพิมพ์ ฿" sqref="L7:L500" xr:uid="{3DE8EF58-E9D9-4286-A04F-19932AB24964}">
       <formula1>0</formula1>
       <formula2>10000000</formula2>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่เป็นวันที่ ปี ค.ศ. เช่น 20/10/2026" promptTitle="วันที่ Prescreen" prompt="วันที่ HRS คัดกรอง ใส่เป็นวันที่ของ Excel ใช้ปี ค.ศ. เช่น 20/10/2026" sqref="M7:M500" xr:uid="{0C7FDED1-0323-44EB-B09D-2123EAF1043A}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่เป็นวันที่ ปี ค.ศ. เช่น 20/10/2026" promptTitle="วันที่ Prescreen" prompt="วันที่ HRS คัดกรอง ใส่เป็นวันที่ของ Excel ใช้ปี ค.ศ. เช่น 20/10/2026" sqref="M7:M500" xr:uid="{D7F29612-C8F7-46DB-9129-3ED08969061F}">
       <formula1>DATE(2000,1,1)</formula1>
       <formula2>DATE(2100,12,31)</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="เลือกจากรายการเท่านั้น" promptTitle="HR Recommendation" prompt="เลือกจากรายการ: แนะนำอย่างยิ่ง / แนะนำ / ควรพิจารณา / ทบทวน · เว้นว่าง = ระบบเลือกให้จาก Candidate Score" sqref="N7:N500" xr:uid="{0C87C4CE-0A3C-40EA-93B3-73A2F8AB4126}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="เลือกจากรายการเท่านั้น" promptTitle="HR Recommendation" prompt="เลือกจากรายการ: แนะนำอย่างยิ่ง / แนะนำ / ควรพิจารณา / ทบทวน · เว้นว่าง = ระบบเลือกให้จาก Candidate Score" sqref="N7:N500" xr:uid="{1D390D52-0E9E-4100-9E36-E763E4CA3AA0}">
       <formula1>"แนะนำอย่างยิ่ง,แนะนำ,ควรพิจารณา,ทบทวน"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="HR Highlight" prompt="ความเห็นของ HRS จุดเด่นหรือข้อสังเกต แสดงบนการ์ดผู้สมัครให้แผนกเห็น" sqref="O7:O500" xr:uid="{3F580D42-362B-4DF1-86E8-2CF41B1B341C}"/>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขจำนวนเต็ม 1 ถึง 5 หรือเว้นว่าง" promptTitle="คะแนน ประสบการณ์" prompt="บริษัท ประเภทธุรกิจ ตำแหน่ง ระยะเวลา ขนาดงาน และขอบเขตความรับผิดชอบ · ใส่ 1–5" sqref="P7:P500" xr:uid="{B601FD9A-D226-4F27-9CAB-D4BE719C4C8C}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="HR Highlight" prompt="ความเห็นของ HRS จุดเด่นหรือข้อสังเกต แสดงบนการ์ดผู้สมัครให้แผนกเห็น" sqref="O7:O500" xr:uid="{E5F813E0-6EA0-43B9-BD4C-83156C5CE6B9}"/>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขจำนวนเต็ม 1 ถึง 5 หรือเว้นว่าง" promptTitle="คะแนน ประสบการณ์" prompt="บริษัท ประเภทธุรกิจ ตำแหน่ง ระยะเวลา ขนาดงาน และขอบเขตความรับผิดชอบ · ใส่ 1–5" sqref="P7:P500" xr:uid="{60B0037F-DA7A-468A-9E8B-9CF7CDA1BFCA}">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขจำนวนเต็ม 1 ถึง 5 หรือเว้นว่าง" promptTitle="คะแนน ความรู้และทักษะ" prompt="ความรู้เฉพาะทาง โปรแกรม เครื่องมือ ระบบ ภาษา และตัวอย่างการใช้งาน · ใส่ 1–5" sqref="Q7:Q500" xr:uid="{B2D1D225-A5DC-4A1A-A03E-44A532E2681B}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขจำนวนเต็ม 1 ถึง 5 หรือเว้นว่าง" promptTitle="คะแนน ความรู้และทักษะ" prompt="ความรู้เฉพาะทาง โปรแกรม เครื่องมือ ระบบ ภาษา และตัวอย่างการใช้งาน · ใส่ 1–5" sqref="Q7:Q500" xr:uid="{D5F73730-24FB-4842-ABA1-402EE7D849CF}">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขจำนวนเต็ม 1 ถึง 5 หรือเว้นว่าง" promptTitle="คะแนน ผลงาน" prompt="โครงการ รางวัล บทบาทที่ลงมือทำ และผลลัพธ์ที่เป็นตัวเลขหรือคุณภาพ · ใส่ 1–5" sqref="R7:R500" xr:uid="{20033818-177B-4D74-BE32-2A35F85376C0}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขจำนวนเต็ม 1 ถึง 5 หรือเว้นว่าง" promptTitle="คะแนน ผลงาน" prompt="โครงการ รางวัล บทบาทที่ลงมือทำ และผลลัพธ์ที่เป็นตัวเลขหรือคุณภาพ · ใส่ 1–5" sqref="R7:R500" xr:uid="{D80746AC-6A53-482C-8A19-FEB6617950F1}">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขจำนวนเต็ม 1 ถึง 5 หรือเว้นว่าง" promptTitle="คะแนน เส้นทางอาชีพ" prompt="ลำดับงาน วันเริ่ม–สิ้นสุด การเลื่อนตำแหน่ง และเหตุผลย้ายงาน · ใส่ 1–5" sqref="S7:S500" xr:uid="{517FC630-D9B0-4EE5-BF23-C91A7D39C17E}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขจำนวนเต็ม 1 ถึง 5 หรือเว้นว่าง" promptTitle="คะแนน เส้นทางอาชีพ" prompt="ลำดับงาน วันเริ่ม–สิ้นสุด การเลื่อนตำแหน่ง และเหตุผลย้ายงาน · ใส่ 1–5" sqref="S7:S500" xr:uid="{3E2A565B-181B-4604-85C4-A092249CE8BB}">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขจำนวนเต็ม 1 ถึง 5 หรือเว้นว่าง" promptTitle="คะแนน การเรียนรู้" prompt="การศึกษา ใบอนุญาต ใบรับรอง หลักสูตรอบรม และการนำความรู้ไปใช้ · ใส่ 1–5" sqref="T7:T500" xr:uid="{2F82D01E-C1C6-4E09-B234-99EF2AD6B277}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขจำนวนเต็ม 1 ถึง 5 หรือเว้นว่าง" promptTitle="คะแนน การเรียนรู้" prompt="การศึกษา ใบอนุญาต ใบรับรอง หลักสูตรอบรม และการนำความรู้ไปใช้ · ใส่ 1–5" sqref="T7:T500" xr:uid="{9ED5D375-11BF-434B-906D-7E0142193183}">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขจำนวนเต็ม 1 ถึง 5 หรือเว้นว่าง" promptTitle="คะแนน ความน่าเชื่อถือ" prompt="ความสอดคล้องของวันที่ ตำแหน่ง ตัวเลข ผลงาน และหลักฐานใน Resume · ใส่ 1–5" sqref="U7:U500" xr:uid="{E0B15059-B89A-4A5E-97E6-5F016B1C4252}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขจำนวนเต็ม 1 ถึง 5 หรือเว้นว่าง" promptTitle="คะแนน ความน่าเชื่อถือ" prompt="ความสอดคล้องของวันที่ ตำแหน่ง ตัวเลข ผลงาน และหลักฐานใน Resume · ใส่ 1–5" sqref="U7:U500" xr:uid="{93113A97-A0E4-47D3-9D2C-3478788587A9}">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขจำนวนเต็ม 1 ถึง 5 หรือเว้นว่าง" promptTitle="คะแนน Tech &amp; AI" prompt="เครื่องมือดิจิทัล ระบบอัตโนมัติ หรือ AI ที่ใช้กับงานจริง พร้อมบทบาทและผลลัพธ์ · ใส่ 1–5" sqref="V7:V500" xr:uid="{AE9A4C06-90D0-45D0-B2F8-34F9080200DC}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่ตัวเลขจำนวนเต็ม 1 ถึง 5 หรือเว้นว่าง" promptTitle="คะแนน Tech &amp; AI" prompt="เครื่องมือดิจิทัล ระบบอัตโนมัติ หรือ AI ที่ใช้กับงานจริง พร้อมบทบาทและผลลัพธ์ · ใส่ 1–5" sqref="V7:V500" xr:uid="{DEF38040-1EDD-4099-8144-CB7EA7AF177B}">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="เลือกจากรายการเท่านั้น" promptTitle="Executive Decision" prompt="เลือกจากรายการ · เว้นว่าง = รอพิจารณา" sqref="W7:W500" xr:uid="{0EE0FB11-EAC6-4520-84B1-92C7C820A127}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="เลือกจากรายการเท่านั้น" promptTitle="Executive Decision" prompt="เลือกจากรายการ · เว้นว่าง = รอพิจารณา" sqref="W7:W500" xr:uid="{855E1903-42E6-45C1-B17D-A98E0EC7F72D}">
       <formula1>"รอพิจารณา,เรียกสัมภาษณ์,นัดสัมภาษณ์แล้ว,สำรอง,ไม่พิจารณา"</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่วันและเวลา ปี ค.ศ. เช่น 10/11/2026 10:00" promptTitle="วัน/เวลา ที่ต้องการนัดสัมภาษณ์" prompt="ไม่บังคับ ใส่วันและเวลา เช่น 10/11/2026 10:00 (ปี ค.ศ.) ระบบบันทึกเป็นนัด Onsite · ถ้า Executive Decision = นัดสัมภาษณ์แล้ว จะถือว่ายืนยันแล้ว" sqref="X7:X500" xr:uid="{5F14F21C-8FAB-4770-B732-343B13B23572}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="ใส่วันและเวลา ปี ค.ศ. เช่น 10/11/2026 10:00" promptTitle="วัน/เวลา ที่ต้องการนัดสัมภาษณ์" prompt="ไม่บังคับ ใส่วันและเวลา เช่น 10/11/2026 10:00 (ปี ค.ศ.) ระบบบันทึกเป็นนัด Onsite · ถ้า Executive Decision = นัดสัมภาษณ์แล้ว จะถือว่ายืนยันแล้ว" sqref="X7:X500" xr:uid="{78BA56E0-2B35-4668-B6E5-2EC4FAFCC0C3}">
       <formula1>DATE(2000,1,1)</formula1>
       <formula2>DATE(2100,12,31)</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="ชื่อผู้สัมภาษณ์" prompt="ชื่อผู้สัมภาษณ์ 1 คน เพิ่มตำแหน่ง ฝ่าย และคนอื่นได้ภายหลังในระบบ" sqref="Y7:Y500" xr:uid="{621D4900-260A-4EB9-9D73-A407619362AF}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="หน่วยงาน/โครงการ" prompt="เว้นว่าง = อยู่ใน Candidate Pool · ใส่รหัสแผนกที่มีในระบบ (เช่น ENG-01) = ส่งเข้า Pool ของแผนกนั้นทันที · Return to HR = คืนเข้า Candidate Pool" sqref="Z7:Z500" xr:uid="{41329FF2-212B-47D5-8E03-68FB2BF8961A}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="ชื่อโครงการ" prompt="ชื่อโครงการที่จะให้ผู้สมัครไปประจำ (ถ้ามี)" sqref="AA7:AA500" xr:uid="{32AFC0BD-9E0C-43F2-ACD1-42F3F024E730}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="หมายเหตุ" prompt="ข้อความเพิ่มเติมอื่นๆ" sqref="AB7:AB500" xr:uid="{8EEFAD6A-1E51-4CBC-8D0E-2C2D48EF2585}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="ชื่อผู้สัมภาษณ์" prompt="ชื่อผู้สัมภาษณ์ 1 คน เพิ่มตำแหน่ง ฝ่าย และคนอื่นได้ภายหลังในระบบ" sqref="Y7:Y500" xr:uid="{49B7737B-F7DA-431F-9841-60E9ED56FDAE}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="หน่วยงาน/โครงการ" prompt="เว้นว่าง = อยู่ใน Candidate Pool · ใส่รหัสแผนกที่มีในระบบ (เช่น ENG-01) = ส่งเข้า Pool ของแผนกนั้นทันที · Return to HR = คืนเข้า Candidate Pool" sqref="Z7:Z500" xr:uid="{D5C92ED6-E3C3-44F4-BA29-71231A72229A}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="ชื่อโครงการ" prompt="ชื่อโครงการที่จะให้ผู้สมัครไปประจำ (ถ้ามี)" sqref="AA7:AA500" xr:uid="{5321EEA2-4C48-4457-95C8-6D8CBEAA9E3D}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="หมายเหตุ" prompt="ข้อความเพิ่มเติมอื่นๆ" sqref="AB7:AB500" xr:uid="{385B351C-A3FC-4BC3-8C30-04E058F087C3}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF021C2C-B318-4604-8933-66C58B594FC0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D47299C9-D44C-468C-9367-CD854D9C1177}">
   <dimension ref="A1:E42"/>
   <sheetFormatPr defaultRowHeight="16.8"/>
   <cols>
@@ -10984,15 +10966,15 @@
   <sheetData>
     <row r="1" spans="1:5" ht="34.049999999999997" customHeight="1">
       <c r="A1" s="24" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="30" customHeight="1">
       <c r="A3" s="25" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C3" s="26"/>
       <c r="D3" s="26"/>
@@ -11000,10 +10982,10 @@
     </row>
     <row r="4" spans="1:5" ht="30" customHeight="1">
       <c r="A4" s="25" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C4" s="26"/>
       <c r="D4" s="26"/>
@@ -11011,21 +10993,21 @@
     </row>
     <row r="5" spans="1:5" ht="30" customHeight="1">
       <c r="A5" s="25" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C5" s="26"/>
       <c r="D5" s="26"/>
       <c r="E5" s="26"/>
     </row>
-    <row r="6" spans="1:5" ht="30" customHeight="1">
+    <row r="6" spans="1:5" ht="48" customHeight="1">
       <c r="A6" s="25" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C6" s="26"/>
       <c r="D6" s="26"/>
@@ -11033,10 +11015,10 @@
     </row>
     <row r="7" spans="1:5" ht="48" customHeight="1">
       <c r="A7" s="25" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C7" s="26"/>
       <c r="D7" s="26"/>
@@ -11044,10 +11026,10 @@
     </row>
     <row r="8" spans="1:5" ht="48" customHeight="1">
       <c r="A8" s="25" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C8" s="26"/>
       <c r="D8" s="26"/>
@@ -11055,10 +11037,10 @@
     </row>
     <row r="9" spans="1:5" ht="30" customHeight="1">
       <c r="A9" s="25" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C9" s="26"/>
       <c r="D9" s="26"/>
@@ -11066,10 +11048,10 @@
     </row>
     <row r="10" spans="1:5" ht="30" customHeight="1">
       <c r="A10" s="25" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C10" s="26"/>
       <c r="D10" s="26"/>
@@ -11077,10 +11059,10 @@
     </row>
     <row r="11" spans="1:5" ht="30" customHeight="1">
       <c r="A11" s="25" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C11" s="26"/>
       <c r="D11" s="26"/>
@@ -11088,10 +11070,10 @@
     </row>
     <row r="12" spans="1:5" ht="30" customHeight="1">
       <c r="A12" s="25" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C12" s="26"/>
       <c r="D12" s="26"/>
@@ -11099,443 +11081,441 @@
     </row>
     <row r="14" spans="1:5" ht="50.4">
       <c r="A14" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="B14" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="C14" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="D14" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="E14" s="27" t="s">
         <v>118</v>
-      </c>
-      <c r="B14" s="27" t="s">
-        <v>104</v>
-      </c>
-      <c r="C14" s="27" t="s">
-        <v>119</v>
-      </c>
-      <c r="D14" s="27" t="s">
-        <v>120</v>
-      </c>
-      <c r="E14" s="27" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="33.6">
       <c r="A15" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="29" t="s">
-        <v>104</v>
-      </c>
+      <c r="B15" s="28"/>
       <c r="C15" s="28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D15" s="28" t="s">
-        <v>123</v>
-      </c>
-      <c r="E15" s="30" t="s">
-        <v>11</v>
+        <v>9</v>
+      </c>
+      <c r="E15" s="29" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" s="29" t="s">
-        <v>104</v>
+        <v>12</v>
+      </c>
+      <c r="B16" s="30" t="s">
+        <v>101</v>
       </c>
       <c r="C16" s="28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D16" s="28" t="s">
-        <v>124</v>
-      </c>
-      <c r="E16" s="30" t="s">
-        <v>16</v>
+        <v>121</v>
+      </c>
+      <c r="E16" s="29" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="28" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B17" s="28"/>
       <c r="C17" s="28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="E17" s="30" t="s">
-        <v>21</v>
+        <v>16</v>
+      </c>
+      <c r="E17" s="29" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="33.6">
       <c r="A18" s="28" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B18" s="28"/>
       <c r="C18" s="28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D18" s="28" t="s">
-        <v>24</v>
-      </c>
-      <c r="E18" s="30" t="s">
-        <v>26</v>
+        <v>21</v>
+      </c>
+      <c r="E18" s="29" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="28" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B19" s="28"/>
       <c r="C19" s="28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D19" s="28" t="s">
-        <v>29</v>
-      </c>
-      <c r="E19" s="30" t="s">
-        <v>31</v>
+        <v>26</v>
+      </c>
+      <c r="E19" s="29" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="28" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B20" s="28"/>
       <c r="C20" s="28" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="D20" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="E20" s="30" t="s">
-        <v>126</v>
+        <v>31</v>
+      </c>
+      <c r="E20" s="29" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="28" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B21" s="28"/>
       <c r="C21" s="28" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="D21" s="28" t="s">
-        <v>36</v>
-      </c>
-      <c r="E21" s="30" t="s">
-        <v>127</v>
+        <v>33</v>
+      </c>
+      <c r="E21" s="29" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="28" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B22" s="28"/>
       <c r="C22" s="28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D22" s="28" t="s">
-        <v>38</v>
-      </c>
-      <c r="E22" s="30" t="s">
-        <v>40</v>
+        <v>35</v>
+      </c>
+      <c r="E22" s="29" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="28" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B23" s="28"/>
       <c r="C23" s="28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>43</v>
-      </c>
-      <c r="E23" s="30" t="s">
-        <v>45</v>
+        <v>40</v>
+      </c>
+      <c r="E23" s="29" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="33.6">
       <c r="A24" s="28" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B24" s="28"/>
       <c r="C24" s="28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D24" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="E24" s="30" t="s">
-        <v>50</v>
+        <v>45</v>
+      </c>
+      <c r="E24" s="29" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="33.6">
       <c r="A25" s="28" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B25" s="28"/>
       <c r="C25" s="28" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D25" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="E25" s="30" t="s">
-        <v>129</v>
+        <v>49</v>
+      </c>
+      <c r="E25" s="29" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="28" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B26" s="28"/>
       <c r="C26" s="28" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D26" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="E26" s="30" t="s">
-        <v>130</v>
+        <v>51</v>
+      </c>
+      <c r="E26" s="29" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="28" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B27" s="28"/>
       <c r="C27" s="28" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="E27" s="30" t="s">
-        <v>131</v>
+        <v>53</v>
+      </c>
+      <c r="E27" s="29" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="33.6">
       <c r="A28" s="28" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B28" s="28"/>
       <c r="C28" s="28" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D28" s="28" t="s">
-        <v>58</v>
-      </c>
-      <c r="E28" s="30" t="s">
-        <v>60</v>
+        <v>55</v>
+      </c>
+      <c r="E28" s="29" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="33.6">
       <c r="A29" s="28" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B29" s="28"/>
       <c r="C29" s="28" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D29" s="28" t="s">
-        <v>63</v>
-      </c>
-      <c r="E29" s="30" t="s">
-        <v>65</v>
+        <v>60</v>
+      </c>
+      <c r="E29" s="29" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="33.6">
       <c r="A30" s="28" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B30" s="28"/>
       <c r="C30" s="28" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D30" s="28" t="s">
-        <v>135</v>
-      </c>
-      <c r="E30" s="30" t="s">
-        <v>136</v>
+        <v>132</v>
+      </c>
+      <c r="E30" s="29" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="33.6">
       <c r="A31" s="28" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B31" s="28"/>
       <c r="C31" s="28" t="s">
+        <v>131</v>
+      </c>
+      <c r="D31" s="28" t="s">
         <v>134</v>
       </c>
-      <c r="D31" s="28" t="s">
-        <v>137</v>
-      </c>
-      <c r="E31" s="30" t="s">
-        <v>138</v>
+      <c r="E31" s="29" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="33.6">
       <c r="A32" s="28" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B32" s="28"/>
       <c r="C32" s="28" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D32" s="28" t="s">
-        <v>139</v>
-      </c>
-      <c r="E32" s="30" t="s">
         <v>136</v>
+      </c>
+      <c r="E32" s="29" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="28" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B33" s="28"/>
       <c r="C33" s="28" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D33" s="28" t="s">
-        <v>140</v>
-      </c>
-      <c r="E33" s="30" t="s">
-        <v>138</v>
+        <v>137</v>
+      </c>
+      <c r="E33" s="29" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="33.6">
       <c r="A34" s="28" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B34" s="28"/>
       <c r="C34" s="28" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D34" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="E34" s="30" t="s">
         <v>138</v>
+      </c>
+      <c r="E34" s="29" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="33.6">
       <c r="A35" s="28" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B35" s="28"/>
       <c r="C35" s="28" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D35" s="28" t="s">
-        <v>142</v>
-      </c>
-      <c r="E35" s="30" t="s">
-        <v>138</v>
+        <v>139</v>
+      </c>
+      <c r="E35" s="29" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="33.6">
       <c r="A36" s="28" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B36" s="28"/>
       <c r="C36" s="28" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D36" s="28" t="s">
-        <v>143</v>
-      </c>
-      <c r="E36" s="30" t="s">
-        <v>136</v>
+        <v>140</v>
+      </c>
+      <c r="E36" s="29" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="28" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B37" s="28"/>
       <c r="C37" s="28" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D37" s="28" t="s">
-        <v>82</v>
-      </c>
-      <c r="E37" s="30" t="s">
-        <v>84</v>
+        <v>79</v>
+      </c>
+      <c r="E37" s="29" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="33.6">
       <c r="A38" s="28" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B38" s="28"/>
       <c r="C38" s="28" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D38" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="E38" s="30" t="s">
-        <v>145</v>
+        <v>83</v>
+      </c>
+      <c r="E38" s="29" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="28" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B39" s="28"/>
       <c r="C39" s="28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D39" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="E39" s="30" t="s">
-        <v>145</v>
+        <v>85</v>
+      </c>
+      <c r="E39" s="29" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="33.6">
       <c r="A40" s="28" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B40" s="28"/>
       <c r="C40" s="28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D40" s="28" t="s">
-        <v>90</v>
-      </c>
-      <c r="E40" s="30" t="s">
-        <v>145</v>
+        <v>87</v>
+      </c>
+      <c r="E40" s="29" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="28" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B41" s="28"/>
       <c r="C41" s="28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D41" s="28" t="s">
-        <v>92</v>
-      </c>
-      <c r="E41" s="30" t="s">
-        <v>145</v>
+        <v>89</v>
+      </c>
+      <c r="E41" s="29" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="28" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B42" s="28"/>
       <c r="C42" s="28" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D42" s="28" t="s">
-        <v>94</v>
-      </c>
-      <c r="E42" s="30" t="s">
-        <v>145</v>
+        <v>91</v>
+      </c>
+      <c r="E42" s="29" t="s">
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>